<commit_message>
test: update guangming and jinjiang retest
</commit_message>
<xml_diff>
--- a/测试/日报及月报发送记录_测试.xlsx
+++ b/测试/日报及月报发送记录_测试.xlsx
@@ -2504,7 +2504,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M119"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="D6" s="29" t="inlineStr">
         <is>
-          <t>累计未发4次</t>
+          <t>累计未发5次</t>
         </is>
       </c>
       <c r="G6" s="31" t="inlineStr">
@@ -2895,7 +2895,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D10" s="33" t="n"/>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>累计迟发1次</t>
+        </is>
+      </c>
       <c r="G10" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3875,6 +3879,72 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
test: update guangzhou retest
</commit_message>
<xml_diff>
--- a/测试/日报及月报发送记录_测试.xlsx
+++ b/测试/日报及月报发送记录_测试.xlsx
@@ -2935,7 +2935,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D11" s="36" t="n"/>
+      <c r="D11" s="36" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="G11" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2971,7 +2975,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D12" s="39" t="n"/>
+      <c r="D12" s="39" t="inlineStr">
+        <is>
+          <t>累计迟发1次</t>
+        </is>
+      </c>
       <c r="G12" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>

</xml_diff>